<commit_message>
Fan Dance times for its real load, in lockstep with the app (2026-10-03)
UKSF Fan Dance Good 3:30 -> 3:55, Excellent 3:15 -> 3:40, Elite 3:00 -> 3:30
(Pass 4:10), changeset 4 of scripts/apply-military-top-tiers-2026-10-02.py.
check:app-ors: 0 differences.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_Operator_Standards.xlsx
+++ b/config/standards/TPF_Operator_Standards.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,10 +563,18 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
           <t>2026-10-03, later (the deadlift Excellent evened out, tpf-app mirror; record: tpf-app docs/build/55_SPECIAL_FORCES_AND_ELITE_UNIT_TIERS.md section 10.1): the owner, shown police at 90 / 115 / 140 / 205 kg, 'Even it out a bit 170kg is barely elite'. On every unit and both bars, Excellent = (Good + Elite) / 2 rounded to the nearest 5 kg (a half rounds up), only ever raised — all 25 deadlift rows here rose; Pass, Good and Elite unchanged. Script: scripts/apply-military-top-tiers-2026-10-02.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-03, latest (the Fan Dance's faster tiers, tpf-app mirror; record: tpf-app docs/build/55_SPECIAL_FORCES_AND_ELITE_UNIT_TIERS.md section 11.1): told the kept 3:00 Elite at the ~23 kg selection load is close to unreachable, the owner: 'adjust times then'. UKSF Fan Dance Good 3:30:00 -&gt; 3:55:00, Excellent 3:15:00 -&gt; 3:40:00, Elite 3:00:00 -&gt; 3:30:00; Pass stays the published 4:10:00. TPF's method (the app's ruck model plus its hilly-terrain band for the ~1,100 m climb), not a source. Script: scripts/apply-military-top-tiers-2026-10-02.py.</t>
         </is>
       </c>
     </row>
@@ -9033,22 +9041,22 @@
       </c>
       <c r="H162" t="inlineStr">
         <is>
+          <t>3:55:00</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>3:40:00</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
           <t>3:30:00</t>
         </is>
       </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>3:15:00</t>
-        </is>
-      </c>
-      <c r="J162" t="inlineStr">
-        <is>
-          <t>3:00:00</t>
-        </is>
-      </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>ORS (tpf-app mirror 2026-07-16); The selection load and its published cut-off (the owner, 2026-10-02: 'Fan dance should be with proper weight'): renamed from 'Fan Dance (24 km @ 35 lb + rifle) — optional'; Pass 4:00:00 -&gt; 4:10:00; Good, Excellent and Elite kept; the app's cite: 'UKSF selection Fan Dance: 4 h 10 min allowed; 18 kg bergen + rifle + water (third-party accounts)' (plan 55 §10.3); id pinned to 'fan_dance_24_km_35_lb_rifle_optional' so stored results still match — tpf-app mirror 2026-10-03 (plan 55 §10.2)</t>
+          <t>ORS (tpf-app mirror 2026-07-16); The selection load and its published cut-off (the owner, 2026-10-02: 'Fan dance should be with proper weight'): renamed from 'Fan Dance (24 km @ 35 lb + rifle) — optional'; Pass 4:00:00 -&gt; 4:10:00; Good, Excellent and Elite kept; the app's cite: 'UKSF selection Fan Dance: 4 h 10 min allowed; 18 kg bergen + rifle + water (third-party accounts)' (plan 55 §10.3); id pinned to 'fan_dance_24_km_35_lb_rifle_optional' so stored results still match — tpf-app mirror 2026-10-03 (plan 55 §10.2); Good 3:30:00 -&gt; 3:55:00, Excellent 3:15:00 -&gt; 3:40:00, Elite 3:00:00 -&gt; 3:30:00; Pass kept at the published 4:10:00 (the owner, 2026-10-03, told a 3:00 Elite at the ~23 kg selection load is close to unreachable: 'adjust times then'). TPF's method, not a source: the app's ruck model plus its hilly-terrain band (x 1.15) for the ~1,100 m of ascent; Elite 3:30 reads 2:16:38 on the app's 12 mi @ 35 lb scale (inside the special-forces band, between Pararescue and the Rangers) and is slower than the best known 35 lb time (3:14, third-party) carried to 23 kg; Good and Excellent split the 40 minutes 20 : 15 : 15 like the tier percentages, to the nearest 5 min. Label unchanged; the app's cite now reads: 'UKSF selection Fan Dance: 4 h 10 min allowed; 18 kg bergen + rifle + water (third-party accounts). Faster tiers TPF's: the ruck model plus a hilly-terrain climb allowance (plan 55 §11)' — tpf-app mirror 2026-10-03 (plan 55 §11.1)</t>
         </is>
       </c>
       <c r="M162" t="inlineStr">

</xml_diff>